<commit_message>
Update modules 5 & 6
</commit_message>
<xml_diff>
--- a/data/add_students/BSSE_students.xlsx
+++ b/data/add_students/BSSE_students.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,38 +417,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Father's Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Enrollment No</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Seat No</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
@@ -453,17 +457,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hussain Khan</t>
+          <t>Abdul Aziz</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Adeel Khan</t>
+          <t>Farrukh Khan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KU/DCS/439563-2022</t>
+          <t>KU/DCS/439363-2022</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -473,24 +477,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>hussain.khan1@ubit.edu.pk</t>
+          <t>abdul.aziz@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shahzad Baig</t>
+          <t>Adeel Hashmi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Imran Baig</t>
+          <t>Yousuf Hashmi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KU/DCS/258176-2022</t>
+          <t>KU/DCS/538485-2022</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -500,24 +504,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>shahzad.baig2@ubit.edu.pk</t>
+          <t>adeel.hashmi18@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hassan Butt</t>
+          <t>Ahmed Butt</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nasir Butt</t>
+          <t>Waqas Butt</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KU/DCS/514002-2022</t>
+          <t>KU/DCS/961168-2022</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -527,24 +531,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>hassan.butt3@ubit.edu.pk</t>
+          <t>ahmed.butt7@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Waqas Rizvi</t>
+          <t>Ahmed Raza</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Abdul Rizvi</t>
+          <t>Waqas Raza</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KU/DCS/782554-2022</t>
+          <t>KU/DCS/150631-2022</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -554,24 +558,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>waqas.rizvi4@ubit.edu.pk</t>
+          <t>ahmed.raza5@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ahmed Raza</t>
+          <t>Aiman Hashmi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Waqas Raza</t>
+          <t>Zafar Hashmi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KU/DCS/150631-2022</t>
+          <t>KU/DCS/325127-2022</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -581,24 +585,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ahmed.raza5@ubit.edu.pk</t>
+          <t>aiman.hashmi14@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Danish Awan</t>
+          <t>Ali Chaudhry</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Zafar Awan</t>
+          <t>Aziz Chaudhry</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KU/DCS/175954-2022</t>
+          <t>KU/DCS/423466-2022</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -608,24 +612,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>danish.awan6@ubit.edu.pk</t>
+          <t>ali.chaudhry47@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ahmed Butt</t>
+          <t>Ali Malik</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Waqas Butt</t>
+          <t>Naveed Malik</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KU/DCS/961168-2022</t>
+          <t>KU/DCS/483452-2022</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -635,24 +639,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ahmed.butt7@ubit.edu.pk</t>
+          <t>ali.malik10@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nasir Rizvi</t>
+          <t>Ali Shah</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Junaid Rizvi</t>
+          <t>Anwar Shah</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KU/DCS/661913-2022</t>
+          <t>KU/DCS/208061-2022</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -662,24 +666,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>nasir.rizvi8@ubit.edu.pk</t>
+          <t>ali.shah52@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Anum Mirza</t>
+          <t>Amna Baig</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Adeel Mirza</t>
+          <t>Imran Baig</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KU/DCS/198702-2022</t>
+          <t>KU/DCS/331821-2022</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -689,24 +693,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>anum.mirza9@ubit.edu.pk</t>
+          <t>amna.baig37@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ali Malik</t>
+          <t>Amna Farooq</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Naveed Malik</t>
+          <t>Junaid Farooq</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KU/DCS/483452-2022</t>
+          <t>KU/DCS/698951-2022</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -716,24 +720,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ali.malik10@ubit.edu.pk</t>
+          <t>amna.farooq54@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hira Chaudhry</t>
+          <t>Anum Mirza</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Imran Chaudhry</t>
+          <t>Adeel Mirza</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KU/DCS/711097-2022</t>
+          <t>KU/DCS/198702-2022</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -743,24 +747,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>hira.chaudhry11@ubit.edu.pk</t>
+          <t>anum.mirza9@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rayyan Iqbal</t>
+          <t>Areeba Khan</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tariq Iqbal</t>
+          <t>Tariq Khan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KU/DCS/160816-2022</t>
+          <t>KU/DCS/709851-2022</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -770,24 +774,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>rayyan.iqbal12@ubit.edu.pk</t>
+          <t>areeba.khan53@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Usman Abbasi</t>
+          <t>Asif Mirza</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tariq Abbasi</t>
+          <t>Saleem Mirza</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KU/DCS/632084-2022</t>
+          <t>KU/DCS/429407-2022</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -797,24 +801,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>usman.abbasi13@ubit.edu.pk</t>
+          <t>asif.mirza71@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aiman Hashmi</t>
+          <t>Ayesha Ahmed</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Zafar Hashmi</t>
+          <t>Rashid Ahmed</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KU/DCS/325127-2022</t>
+          <t>KU/DCS/139317-2022</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -824,24 +828,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>aiman.hashmi14@ubit.edu.pk</t>
+          <t>ayesha.ahmed15@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ayesha Ahmed</t>
+          <t>Ayesha Butt</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Rashid Ahmed</t>
+          <t>Muhammad Butt</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KU/DCS/139317-2022</t>
+          <t>KU/DCS/251262-2022</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -851,24 +855,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ayesha.ahmed15@ubit.edu.pk</t>
+          <t>ayesha.butt43@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nasir Siddiqui</t>
+          <t>Danish Ahmed</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shakeel Siddiqui</t>
+          <t>Anwar Ahmed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KU/DCS/190122-2022</t>
+          <t>KU/DCS/761259-2022</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -878,24 +882,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>nasir.siddiqui16@ubit.edu.pk</t>
+          <t>danish.ahmed29@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Usman Butt</t>
+          <t>Danish Awan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sidra Butt</t>
+          <t>Zafar Awan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>KU/DCS/554710-2022</t>
+          <t>KU/DCS/175954-2022</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -905,24 +909,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>usman.butt17@ubit.edu.pk</t>
+          <t>danish.awan6@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Adeel Hashmi</t>
+          <t>Danish Farooq</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yousuf Hashmi</t>
+          <t>Nasir Farooq</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>KU/DCS/538485-2022</t>
+          <t>KU/DCS/352353-2022</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -932,24 +936,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>adeel.hashmi18@ubit.edu.pk</t>
+          <t>danish.farooq20@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Faizan Raza</t>
+          <t>Danish Iqbal</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Abdul Raza</t>
+          <t>Abdul Iqbal</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KU/DCS/173248-2022</t>
+          <t>KU/DCS/334083-2022</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -959,24 +963,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>faizan.raza19@ubit.edu.pk</t>
+          <t>danish.iqbal28@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Danish Farooq</t>
+          <t>Danish Siddiqui</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nasir Farooq</t>
+          <t>Shakeel Siddiqui</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KU/DCS/352353-2022</t>
+          <t>KU/DCS/195119-2022</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -986,24 +990,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>danish.farooq20@ubit.edu.pk</t>
+          <t>danish.siddiqui21@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Danish Siddiqui</t>
+          <t>Fahad Baig</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Shakeel Siddiqui</t>
+          <t>Aslam Baig</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>KU/DCS/195119-2022</t>
+          <t>KU/DCS/713984-2022</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1013,24 +1017,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>danish.siddiqui21@ubit.edu.pk</t>
+          <t>fahad.baig34@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sara Soomro</t>
+          <t>Fahad Bhatti</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Rafiq Soomro</t>
+          <t>Aslam Bhatti</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>KU/DCS/677814-2022</t>
+          <t>KU/DCS/202163-2022</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1040,24 +1044,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>sara.soomro22@ubit.edu.pk</t>
+          <t>fahad.bhatti58@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Talha Hashmi</t>
+          <t>Faizan Raza</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rafiq Hashmi</t>
+          <t>Abdul Raza</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>KU/DCS/545140-2022</t>
+          <t>KU/DCS/173248-2022</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1067,24 +1071,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>talha.hashmi23@ubit.edu.pk</t>
+          <t>faizan.raza19@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rayyan Chaudhry</t>
+          <t>Faizan Sheikh</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nasir Chaudhry</t>
+          <t>Rafiq Sheikh</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KU/DCS/161981-2022</t>
+          <t>KU/DCS/815131-2022</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1094,24 +1098,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>rayyan.chaudhry24@ubit.edu.pk</t>
+          <t>faizan.sheikh50@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Junaid Malik</t>
+          <t>Faizan Siddiqui</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aslam Malik</t>
+          <t>Tariq Siddiqui</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>KU/DCS/967017-2022</t>
+          <t>KU/DCS/714006-2022</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1121,24 +1125,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>junaid.malik25@ubit.edu.pk</t>
+          <t>faizan.siddiqui73@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Shahzad Malik</t>
+          <t>Fatima Awan</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rashid Malik</t>
+          <t>Zafar Awan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>KU/DCS/692921-2022</t>
+          <t>KU/DCS/955770-2022</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1148,24 +1152,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>shahzad.malik26@ubit.edu.pk</t>
+          <t>fatima.awan49@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sana Chaudhry</t>
+          <t>Hamza Baig</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aslam Chaudhry</t>
+          <t>Yousuf Baig</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>KU/DCS/229815-2022</t>
+          <t>KU/DCS/769949-2022</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1175,24 +1179,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>sana.chaudhry27@ubit.edu.pk</t>
+          <t>hamza.baig55@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Danish Iqbal</t>
+          <t>Hamza Siddiqui</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Abdul Iqbal</t>
+          <t>Imran Siddiqui</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KU/DCS/334083-2022</t>
+          <t>KU/DCS/683705-2022</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1202,24 +1206,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>danish.iqbal28@ubit.edu.pk</t>
+          <t>hamza.siddiqui39@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Danish Ahmed</t>
+          <t>Hassan Ahmed</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Anwar Ahmed</t>
+          <t>Shakeel Ahmed</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>KU/DCS/761259-2022</t>
+          <t>KU/DCS/414328-2022</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1229,24 +1233,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>danish.ahmed29@ubit.edu.pk</t>
+          <t>hassan.ahmed76@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Rabia Chaudhry</t>
+          <t>Hassan Butt</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nasir Chaudhry</t>
+          <t>Nasir Butt</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>KU/DCS/757911-2022</t>
+          <t>KU/DCS/514002-2022</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1256,24 +1260,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>rabia.chaudhry30@ubit.edu.pk</t>
+          <t>hassan.butt3@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rayyan Mirza</t>
+          <t>Hira Chaudhry</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Anwar Mirza</t>
+          <t>Imran Chaudhry</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>KU/DCS/711316-2022</t>
+          <t>KU/DCS/711097-2022</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1283,24 +1287,24 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>rayyan.mirza31@ubit.edu.pk</t>
+          <t>hira.chaudhry11@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Rayyan Bhatti</t>
+          <t>Hira Raza</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Shakeel Bhatti</t>
+          <t>Aziz Raza</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>KU/DCS/164867-2022</t>
+          <t>KU/DCS/657549-2022</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1310,24 +1314,24 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>rayyan.bhatti32@ubit.edu.pk</t>
+          <t>hira.raza68@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Nimra Sheikh</t>
+          <t>Hira Siddiqui</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Adeel Sheikh</t>
+          <t>Sidra Siddiqui</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KU/DCS/705136-2022</t>
+          <t>KU/DCS/223514-2022</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1337,24 +1341,24 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>nimra.sheikh33@ubit.edu.pk</t>
+          <t>hira.siddiqui45@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Fahad Baig</t>
+          <t>Hussain Butt</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Aslam Baig</t>
+          <t>Adeel Butt</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KU/DCS/713984-2022</t>
+          <t>KU/DCS/666950-2022</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1364,24 +1368,24 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>fahad.baig34@ubit.edu.pk</t>
+          <t>hussain.butt44@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Nasir Chaudhry</t>
+          <t>Hussain Khan</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yousuf Chaudhry</t>
+          <t>Adeel Khan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>KU/DCS/515949-2022</t>
+          <t>KU/DCS/439563-2022</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1391,24 +1395,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>nasir.chaudhry35@ubit.edu.pk</t>
+          <t>hussain.khan1@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Mahnoor Mirza</t>
+          <t>Imran Siddiqui</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Shakeel Mirza</t>
+          <t>Abdul Siddiqui</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KU/DCS/151998-2022</t>
+          <t>KU/DCS/832948-2022</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1418,24 +1422,24 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>mahnoor.mirza36@ubit.edu.pk</t>
+          <t>imran.siddiqui80@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Amna Baig</t>
+          <t>Iqra Soomro</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Imran Baig</t>
+          <t>Abdul Soomro</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>KU/DCS/331821-2022</t>
+          <t>KU/DCS/479146-2022</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1445,24 +1449,24 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>amna.baig37@ubit.edu.pk</t>
+          <t>iqra.soomro75@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kamran Bhatti</t>
+          <t>Junaid Malik</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nasir Bhatti</t>
+          <t>Aslam Malik</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>KU/DCS/148845-2022</t>
+          <t>KU/DCS/967017-2022</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1472,24 +1476,24 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>kamran.bhatti38@ubit.edu.pk</t>
+          <t>junaid.malik25@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hamza Siddiqui</t>
+          <t>Junaid Rizvi</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Imran Siddiqui</t>
+          <t>Waqas Rizvi</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KU/DCS/683705-2022</t>
+          <t>KU/DCS/846702-2022</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1499,24 +1503,24 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>hamza.siddiqui39@ubit.edu.pk</t>
+          <t>junaid.rizvi60@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Talha Rizvi</t>
+          <t>Junaid Soomro</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Zafar Rizvi</t>
+          <t>Aziz Soomro</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>KU/DCS/239643-2022</t>
+          <t>KU/DCS/539499-2022</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1526,24 +1530,24 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>talha.rizvi40@ubit.edu.pk</t>
+          <t>junaid.soomro42@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Zain Abbasi</t>
+          <t>Kamran Bhatti</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Shakeel Abbasi</t>
+          <t>Nasir Bhatti</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>KU/DCS/403677-2022</t>
+          <t>KU/DCS/148845-2022</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1553,24 +1557,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>zain.abbasi41@ubit.edu.pk</t>
+          <t>kamran.bhatti38@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Junaid Soomro</t>
+          <t>Mahnoor Hashmi</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Aziz Soomro</t>
+          <t>Naveed Hashmi</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>KU/DCS/539499-2022</t>
+          <t>KU/DCS/575198-2022</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1580,24 +1584,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>junaid.soomro42@ubit.edu.pk</t>
+          <t>mahnoor.hashmi74@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ayesha Butt</t>
+          <t>Mahnoor Malik</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Muhammad Butt</t>
+          <t>Rashid Malik</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>KU/DCS/251262-2022</t>
+          <t>KU/DCS/698646-2022</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1607,24 +1611,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ayesha.butt43@ubit.edu.pk</t>
+          <t>mahnoor.malik46@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hussain Butt</t>
+          <t>Mahnoor Mirza</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Adeel Butt</t>
+          <t>Shakeel Mirza</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>KU/DCS/666950-2022</t>
+          <t>KU/DCS/151998-2022</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1634,24 +1638,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>hussain.butt44@ubit.edu.pk</t>
+          <t>mahnoor.mirza36@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Hira Siddiqui</t>
+          <t>Nasir Chaudhry</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Sidra Siddiqui</t>
+          <t>Yousuf Chaudhry</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>KU/DCS/223514-2022</t>
+          <t>KU/DCS/515949-2022</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1661,24 +1665,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>hira.siddiqui45@ubit.edu.pk</t>
+          <t>nasir.chaudhry35@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Mahnoor Malik</t>
+          <t>Nasir Qureshi</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Rashid Malik</t>
+          <t>Sidra Qureshi</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>KU/DCS/698646-2022</t>
+          <t>KU/DCS/165839-2022</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1688,24 +1692,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>mahnoor.malik46@ubit.edu.pk</t>
+          <t>nasir.qureshi61@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ali Chaudhry</t>
+          <t>Nasir Rizvi</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Aziz Chaudhry</t>
+          <t>Junaid Rizvi</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>KU/DCS/423466-2022</t>
+          <t>KU/DCS/661913-2022</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1715,24 +1719,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ali.chaudhry47@ubit.edu.pk</t>
+          <t>nasir.rizvi8@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Saad Awan</t>
+          <t>Nasir Siddiqui</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Tariq Awan</t>
+          <t>Shakeel Siddiqui</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>KU/DCS/687472-2022</t>
+          <t>KU/DCS/190122-2022</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1742,24 +1746,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>saad.awan48@ubit.edu.pk</t>
+          <t>nasir.siddiqui16@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Fatima Awan</t>
+          <t>Nasir Soomro</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Zafar Awan</t>
+          <t>Imran Soomro</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>KU/DCS/955770-2022</t>
+          <t>KU/DCS/932967-2022</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1769,24 +1773,24 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>fatima.awan49@ubit.edu.pk</t>
+          <t>nasir.soomro78@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Faizan Sheikh</t>
+          <t>Nimra Sheikh</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Rafiq Sheikh</t>
+          <t>Muhammad Bilal Shaikh</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>KU/DCS/815131-2022</t>
+          <t>KU/DCS/705136-2022</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1796,24 +1800,24 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>faizan.sheikh50@ubit.edu.pk</t>
+          <t>nimra.sheikh@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Talha Butt</t>
+          <t>Rabia Chaudhry</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Aziz Butt</t>
+          <t>Nasir Chaudhry</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>KU/DCS/289505-2022</t>
+          <t>KU/DCS/757911-2022</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1823,24 +1827,24 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>talha.butt51@ubit.edu.pk</t>
+          <t>rabia.chaudhry30@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ali Shah</t>
+          <t>Rabia Hashmi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Anwar Shah</t>
+          <t>Rashid Hashmi</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>KU/DCS/208061-2022</t>
+          <t>KU/DCS/691783-2022</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1850,24 +1854,24 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ali.shah52@ubit.edu.pk</t>
+          <t>rabia.hashmi62@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Areeba Khan</t>
+          <t>Rayyan Bhatti</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Tariq Khan</t>
+          <t>Shakeel Bhatti</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>KU/DCS/709851-2022</t>
+          <t>KU/DCS/164867-2022</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1877,24 +1881,24 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>areeba.khan53@ubit.edu.pk</t>
+          <t>rayyan.bhatti32@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Amna Farooq</t>
+          <t>Rayyan Butt</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Junaid Farooq</t>
+          <t>Imran Butt</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>KU/DCS/698951-2022</t>
+          <t>KU/DCS/914983-2022</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1904,24 +1908,24 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>amna.farooq54@ubit.edu.pk</t>
+          <t>rayyan.butt70@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Hamza Baig</t>
+          <t>Rayyan Chaudhry</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yousuf Baig</t>
+          <t>Nasir Chaudhry</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>KU/DCS/769949-2022</t>
+          <t>KU/DCS/161981-2022</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1931,24 +1935,24 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>hamza.baig55@ubit.edu.pk</t>
+          <t>rayyan.chaudhry24@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Usman Raza</t>
+          <t>Rayyan Iqbal</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Saleem Raza</t>
+          <t>Tariq Iqbal</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>KU/DCS/296997-2022</t>
+          <t>KU/DCS/160816-2022</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1958,24 +1962,24 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>usman.raza56@ubit.edu.pk</t>
+          <t>rayyan.iqbal12@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Zain Butt</t>
+          <t>Rayyan Mirza</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Imran Butt</t>
+          <t>Anwar Mirza</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>KU/DCS/490487-2022</t>
+          <t>KU/DCS/711316-2022</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1985,24 +1989,24 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>zain.butt57@ubit.edu.pk</t>
+          <t>rayyan.mirza31@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fahad Bhatti</t>
+          <t>Saad Awan</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Aslam Bhatti</t>
+          <t>Tariq Awan</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>KU/DCS/202163-2022</t>
+          <t>KU/DCS/687472-2022</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2012,24 +2016,24 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>fahad.bhatti58@ubit.edu.pk</t>
+          <t>saad.awan48@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Talha Chaudhry</t>
+          <t>Sana Chaudhry</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Aziz Chaudhry</t>
+          <t>Aslam Chaudhry</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>KU/DCS/674351-2022</t>
+          <t>KU/DCS/229815-2022</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2039,24 +2043,24 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>talha.chaudhry59@ubit.edu.pk</t>
+          <t>sana.chaudhry27@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Junaid Rizvi</t>
+          <t>Sara Soomro</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Waqas Rizvi</t>
+          <t>Rafiq Soomro</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>KU/DCS/846702-2022</t>
+          <t>KU/DCS/677814-2022</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2066,24 +2070,24 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>junaid.rizvi60@ubit.edu.pk</t>
+          <t>sara.soomro22@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Nasir Qureshi</t>
+          <t>Shahzad Baig</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Sidra Qureshi</t>
+          <t>Imran Baig</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>KU/DCS/165839-2022</t>
+          <t>KU/DCS/258176-2022</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2093,24 +2097,24 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>nasir.qureshi61@ubit.edu.pk</t>
+          <t>shahzad.baig2@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Rabia Hashmi</t>
+          <t>Shahzad Bhatti</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Rashid Hashmi</t>
+          <t>Naveed Bhatti</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>KU/DCS/691783-2022</t>
+          <t>KU/DCS/588218-2022</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2120,24 +2124,24 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>rabia.hashmi62@ubit.edu.pk</t>
+          <t>shahzad.bhatti72@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Tariq Soomro</t>
+          <t>Shahzad Chaudhry</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Tariq Soomro</t>
+          <t>Saleem Chaudhry</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>KU/DCS/162496-2022</t>
+          <t>KU/DCS/548363-2022</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2147,24 +2151,24 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>tariq.soomro63@ubit.edu.pk</t>
+          <t>shahzad.chaudhry69@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Zain Iqbal</t>
+          <t>Shahzad Malik</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Muhammad Iqbal</t>
+          <t>Rashid Malik</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>KU/DCS/749078-2022</t>
+          <t>KU/DCS/692921-2022</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2174,24 +2178,24 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>zain.iqbal64@ubit.edu.pk</t>
+          <t>shahzad.malik26@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Waqas Butt</t>
+          <t>Shahzad Qureshi</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Junaid Butt</t>
+          <t>Waqas Qureshi</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>KU/DCS/315963-2022</t>
+          <t>KU/DCS/360494-2022</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2201,24 +2205,24 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>waqas.butt65@ubit.edu.pk</t>
+          <t>shahzad.qureshi77@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Waqas Baig</t>
+          <t>Shahzad Raza</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Muhammad Baig</t>
+          <t>Rashid Raza</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>KU/DCS/620528-2022</t>
+          <t>KU/DCS/288499-2022</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2228,24 +2232,24 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>waqas.baig66@ubit.edu.pk</t>
+          <t>shahzad.raza79@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Zain Ahmed</t>
+          <t>Talha Butt</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Junaid Ahmed</t>
+          <t>Aziz Butt</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>KU/DCS/813451-2022</t>
+          <t>KU/DCS/289505-2022</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2255,24 +2259,24 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>zain.ahmed67@ubit.edu.pk</t>
+          <t>talha.butt51@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Hira Raza</t>
+          <t>Talha Chaudhry</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Aziz Raza</t>
+          <t>Aziz Chaudhry</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>KU/DCS/657549-2022</t>
+          <t>KU/DCS/674351-2022</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2282,24 +2286,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>hira.raza68@ubit.edu.pk</t>
+          <t>talha.chaudhry59@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Shahzad Chaudhry</t>
+          <t>Talha Hashmi</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Saleem Chaudhry</t>
+          <t>Rafiq Hashmi</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>KU/DCS/548363-2022</t>
+          <t>KU/DCS/545140-2022</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2309,24 +2313,24 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>shahzad.chaudhry69@ubit.edu.pk</t>
+          <t>talha.hashmi23@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Rayyan Butt</t>
+          <t>Talha Rizvi</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Imran Butt</t>
+          <t>Zafar Rizvi</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>KU/DCS/914983-2022</t>
+          <t>KU/DCS/239643-2022</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2336,24 +2340,24 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>rayyan.butt70@ubit.edu.pk</t>
+          <t>talha.rizvi40@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Asif Mirza</t>
+          <t>Tariq Soomro</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Saleem Mirza</t>
+          <t>Tariq Soomro</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>KU/DCS/429407-2022</t>
+          <t>KU/DCS/162496-2022</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2363,24 +2367,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>asif.mirza71@ubit.edu.pk</t>
+          <t>tariq.soomro63@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Shahzad Bhatti</t>
+          <t>Usman Abbasi</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Naveed Bhatti</t>
+          <t>Tariq Abbasi</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>KU/DCS/588218-2022</t>
+          <t>KU/DCS/632084-2022</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2390,24 +2394,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>shahzad.bhatti72@ubit.edu.pk</t>
+          <t>usman.abbasi13@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Faizan Siddiqui</t>
+          <t>Usman Butt</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Tariq Siddiqui</t>
+          <t>Sidra Butt</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>KU/DCS/714006-2022</t>
+          <t>KU/DCS/554710-2022</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2417,24 +2421,24 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>faizan.siddiqui73@ubit.edu.pk</t>
+          <t>usman.butt17@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Mahnoor Hashmi</t>
+          <t>Usman Raza</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Naveed Hashmi</t>
+          <t>Saleem Raza</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>KU/DCS/575198-2022</t>
+          <t>KU/DCS/296997-2022</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2444,24 +2448,24 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>mahnoor.hashmi74@ubit.edu.pk</t>
+          <t>usman.raza56@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Iqra Soomro</t>
+          <t>Waqas Baig</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Abdul Soomro</t>
+          <t>Muhammad Baig</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>KU/DCS/479146-2022</t>
+          <t>KU/DCS/620528-2022</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2471,24 +2475,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>iqra.soomro75@ubit.edu.pk</t>
+          <t>waqas.baig66@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Hassan Ahmed</t>
+          <t>Waqas Butt</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Shakeel Ahmed</t>
+          <t>Junaid Butt</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>KU/DCS/414328-2022</t>
+          <t>KU/DCS/315963-2022</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2498,24 +2502,24 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>hassan.ahmed76@ubit.edu.pk</t>
+          <t>waqas.butt65@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Shahzad Qureshi</t>
+          <t>Waqas Rizvi</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Waqas Qureshi</t>
+          <t>Abdul Rizvi</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>KU/DCS/360494-2022</t>
+          <t>KU/DCS/782554-2022</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2525,24 +2529,24 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>shahzad.qureshi77@ubit.edu.pk</t>
+          <t>waqas.rizvi4@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Nasir Soomro</t>
+          <t>Zain Abbasi</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Imran Soomro</t>
+          <t>Shakeel Abbasi</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>KU/DCS/932967-2022</t>
+          <t>KU/DCS/403677-2022</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2552,24 +2556,24 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>nasir.soomro78@ubit.edu.pk</t>
+          <t>zain.abbasi41@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Shahzad Raza</t>
+          <t>Zain Ahmed</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Rashid Raza</t>
+          <t>Junaid Ahmed</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>KU/DCS/288499-2022</t>
+          <t>KU/DCS/813451-2022</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2579,24 +2583,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>shahzad.raza79@ubit.edu.pk</t>
+          <t>zain.ahmed67@ubit.edu.pk</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Imran Siddiqui</t>
+          <t>Zain Butt</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Abdul Siddiqui</t>
+          <t>Imran Butt</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>KU/DCS/832948-2022</t>
+          <t>KU/DCS/490487-2022</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2606,7 +2610,34 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>imran.siddiqui80@ubit.edu.pk</t>
+          <t>zain.butt57@ubit.edu.pk</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Zain Iqbal</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Muhammad Iqbal</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>KU/DCS/749078-2022</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>B22110106081</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>zain.iqbal64@ubit.edu.pk</t>
         </is>
       </c>
     </row>

</xml_diff>